<commit_message>
added couple of new plants and pics
</commit_message>
<xml_diff>
--- a/data/blumen_data.xlsx
+++ b/data/blumen_data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="38280" yWindow="5475" windowWidth="16440" windowHeight="28320" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" state="visible" r:id="rId1"/>
@@ -48,7 +48,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -121,6 +121,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.3999755851924192"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -134,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -166,6 +172,8 @@
     <xf numFmtId="14" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -509,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD5998"/>
+  <dimension ref="A1:AC6062"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14.42578125" customWidth="1" min="1" max="1"/>
@@ -519,40 +527,39 @@
     <col width="15.140625" customWidth="1" min="5" max="6"/>
     <col width="8.5703125" customWidth="1" min="7" max="7"/>
     <col width="11.5703125" customWidth="1" min="8" max="9"/>
-    <col width="11.42578125" customWidth="1" min="10" max="10"/>
-    <col width="74.28515625" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="13"/>
-    <col width="27" customWidth="1" min="14" max="14"/>
-    <col width="42" customWidth="1" min="15" max="15"/>
-    <col width="15.7109375" customWidth="1" min="16" max="16"/>
-    <col width="26.7109375" customWidth="1" min="17" max="17"/>
-    <col width="22.28515625" customWidth="1" min="18" max="18"/>
-    <col width="27.5703125" customWidth="1" min="19" max="19"/>
-    <col width="37.5703125" customWidth="1" min="20" max="21"/>
-    <col width="38.85546875" customWidth="1" min="22" max="22"/>
-    <col width="37" customWidth="1" min="23" max="23"/>
-    <col width="31.5703125" customWidth="1" min="24" max="24"/>
-    <col width="27.85546875" customWidth="1" min="25" max="25"/>
-    <col width="26.42578125" customWidth="1" min="26" max="26"/>
-    <col width="29" customWidth="1" min="27" max="27"/>
-    <col width="37.28515625" customWidth="1" min="28" max="30"/>
-    <col width="36.42578125" customWidth="1" min="31" max="31"/>
-    <col width="28.5703125" customWidth="1" min="32" max="32"/>
-    <col width="30.140625" customWidth="1" min="33" max="34"/>
-    <col width="30.28515625" customWidth="1" min="35" max="35"/>
-    <col width="31" customWidth="1" min="36" max="36"/>
-    <col width="39.140625" customWidth="1" min="37" max="37"/>
-    <col width="41.7109375" customWidth="1" min="38" max="38"/>
-    <col width="39.5703125" customWidth="1" min="39" max="39"/>
-    <col width="29.42578125" customWidth="1" min="40" max="40"/>
-    <col width="30.28515625" customWidth="1" min="41" max="41"/>
-    <col width="25.85546875" customWidth="1" min="42" max="42"/>
-    <col width="30" customWidth="1" min="43" max="43"/>
-    <col width="37.7109375" customWidth="1" min="44" max="44"/>
-    <col width="36" customWidth="1" min="45" max="45"/>
-    <col width="37.7109375" customWidth="1" min="46" max="46"/>
-    <col width="37.28515625" customWidth="1" min="47" max="47"/>
-    <col width="38.5703125" customWidth="1" min="48" max="48"/>
+    <col width="74.28515625" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="12"/>
+    <col width="27" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="15.7109375" customWidth="1" min="15" max="15"/>
+    <col width="26.7109375" customWidth="1" min="16" max="16"/>
+    <col width="22.28515625" customWidth="1" min="17" max="17"/>
+    <col width="27.5703125" customWidth="1" min="18" max="18"/>
+    <col width="37.5703125" customWidth="1" min="19" max="20"/>
+    <col width="38.85546875" customWidth="1" min="21" max="21"/>
+    <col width="37" customWidth="1" min="22" max="22"/>
+    <col width="31.5703125" customWidth="1" min="23" max="23"/>
+    <col width="27.85546875" customWidth="1" min="24" max="24"/>
+    <col width="26.42578125" customWidth="1" min="25" max="25"/>
+    <col width="29" customWidth="1" min="26" max="26"/>
+    <col width="37.28515625" customWidth="1" min="27" max="29"/>
+    <col width="36.42578125" customWidth="1" min="30" max="30"/>
+    <col width="28.5703125" customWidth="1" min="31" max="31"/>
+    <col width="30.140625" customWidth="1" min="32" max="33"/>
+    <col width="30.28515625" customWidth="1" min="34" max="34"/>
+    <col width="31" customWidth="1" min="35" max="35"/>
+    <col width="39.140625" customWidth="1" min="36" max="36"/>
+    <col width="41.7109375" customWidth="1" min="37" max="37"/>
+    <col width="39.5703125" customWidth="1" min="38" max="38"/>
+    <col width="29.42578125" customWidth="1" min="39" max="39"/>
+    <col width="30.28515625" customWidth="1" min="40" max="40"/>
+    <col width="25.85546875" customWidth="1" min="41" max="41"/>
+    <col width="30" customWidth="1" min="42" max="42"/>
+    <col width="37.7109375" customWidth="1" min="43" max="43"/>
+    <col width="36" customWidth="1" min="44" max="44"/>
+    <col width="37.7109375" customWidth="1" min="45" max="45"/>
+    <col width="37.28515625" customWidth="1" min="46" max="46"/>
+    <col width="38.5703125" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1" ht="53.25" customFormat="1" customHeight="1" s="6">
@@ -603,11 +610,6 @@
       </c>
       <c r="J1" s="6" t="inlineStr">
         <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="K1" s="6" t="inlineStr">
-        <is>
           <t>condition</t>
         </is>
       </c>
@@ -624,7 +626,7 @@
       <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="AD2" s="3" t="n"/>
+      <c r="AC2" s="3" t="n"/>
     </row>
     <row r="3" customFormat="1" s="1">
       <c r="A3" s="5" t="n">
@@ -641,7 +643,7 @@
       <c r="D3" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="AD3" s="3" t="n"/>
+      <c r="AC3" s="3" t="n"/>
     </row>
     <row r="4" customFormat="1" s="1">
       <c r="A4" s="5" t="n">
@@ -658,7 +660,7 @@
       <c r="D4" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="AD4" s="3" t="n"/>
+      <c r="AC4" s="3" t="n"/>
     </row>
     <row r="5" customFormat="1" s="1">
       <c r="A5" s="5" t="n">
@@ -675,7 +677,7 @@
       <c r="D5" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="AD5" s="3" t="n"/>
+      <c r="AC5" s="3" t="n"/>
     </row>
     <row r="6" customFormat="1" s="1">
       <c r="A6" s="5" t="n">
@@ -692,7 +694,7 @@
       <c r="D6" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="AD6" s="3" t="n"/>
+      <c r="AC6" s="3" t="n"/>
     </row>
     <row r="7" customFormat="1" s="10">
       <c r="A7" s="8" t="n"/>
@@ -707,8 +709,7 @@
       <c r="L7" s="9" t="n"/>
       <c r="M7" s="9" t="n"/>
       <c r="N7" s="9" t="n"/>
-      <c r="O7" s="9" t="n"/>
-      <c r="AD7" s="11" t="n"/>
+      <c r="AC7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1157,7 +1158,7 @@
       <c r="F44" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K44" s="7" t="inlineStr">
+      <c r="J44" s="7" t="inlineStr">
         <is>
           <t>hat angefangen blätter zu gelben und blätter haben angefangen sich zu krümmen</t>
         </is>
@@ -1244,7 +1245,7 @@
       <c r="F50" t="n">
         <v>1</v>
       </c>
-      <c r="K50" s="7" t="inlineStr">
+      <c r="J50" s="7" t="inlineStr">
         <is>
           <t>hat angefangen blätter zu gelben und blätter haben angefangen sich zu krümmen</t>
         </is>
@@ -1327,7 +1328,7 @@
       <c r="F56" t="n">
         <v>2</v>
       </c>
-      <c r="K56" s="7" t="inlineStr">
+      <c r="J56" s="7" t="inlineStr">
         <is>
           <t>hat angefangen blätter zu gelben und blätter haben angefangen sich zu krümmen</t>
         </is>
@@ -1369,7 +1370,7 @@
       <c r="C58" t="n">
         <v>2</v>
       </c>
-      <c r="K58" s="4" t="inlineStr">
+      <c r="J58" s="4" t="inlineStr">
         <is>
           <t>es hat sich links ein neuer ast angefangen zu bilden</t>
         </is>
@@ -12988,7 +12989,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="K1047" t="inlineStr">
+      <c r="J1047" t="inlineStr">
         <is>
           <t>etwas Spinnmilben</t>
         </is>
@@ -13016,7 +13017,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="K1048" s="7" t="inlineStr">
+      <c r="J1048" s="7" t="inlineStr">
         <is>
           <t>heftige Spinnmilben</t>
         </is>
@@ -17791,7 +17792,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="K1467" t="inlineStr">
+      <c r="J1467" t="inlineStr">
         <is>
           <t>Habe eine Überlebte larve gesehen daher noch mal Pestmix</t>
         </is>
@@ -20927,7 +20928,7 @@
       <c r="D1728" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="K1728" s="7" t="inlineStr">
+      <c r="J1728" s="7" t="inlineStr">
         <is>
           <t>umgepflanzt größeres Gefäß</t>
         </is>
@@ -20956,7 +20957,7 @@
           <t>Peperomia Hope</t>
         </is>
       </c>
-      <c r="K1730" s="7" t="inlineStr">
+      <c r="J1730" s="7" t="inlineStr">
         <is>
           <t>zweiten Zweig dazu gepflanzt</t>
         </is>
@@ -21024,7 +21025,7 @@
       <c r="D1735" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="K1735" s="7" t="inlineStr">
+      <c r="J1735" s="7" t="inlineStr">
         <is>
           <t>umgepflanzt größeres Gefäß</t>
         </is>
@@ -21056,7 +21057,7 @@
       <c r="D1737" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="K1737" s="7" t="inlineStr">
+      <c r="J1737" s="7" t="inlineStr">
         <is>
           <t>umgepflanzt größeres Gefäß</t>
         </is>
@@ -22079,7 +22080,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="K1823" s="7" t="inlineStr">
+      <c r="J1823" s="7" t="inlineStr">
         <is>
           <t>wieder ein wurm nach dem wässern entdeckt</t>
         </is>
@@ -33570,7 +33571,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2828" s="4" t="inlineStr">
+      <c r="J2828" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -33593,7 +33594,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2829" s="4" t="inlineStr">
+      <c r="J2829" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -33677,7 +33678,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2836" s="4" t="inlineStr">
+      <c r="J2836" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -33720,7 +33721,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2839" s="4" t="inlineStr">
+      <c r="J2839" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -33743,7 +33744,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2840" s="4" t="inlineStr">
+      <c r="J2840" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -33776,7 +33777,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2842" s="4" t="inlineStr">
+      <c r="J2842" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -33799,7 +33800,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2843" s="4" t="inlineStr">
+      <c r="J2843" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -33822,7 +33823,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2844" s="4" t="inlineStr">
+      <c r="J2844" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -34246,7 +34247,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2887" s="4" t="inlineStr">
+      <c r="J2887" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -34271,7 +34272,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2888" s="4" t="inlineStr">
+      <c r="J2888" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -34329,7 +34330,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2891" s="4" t="inlineStr">
+      <c r="J2891" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -34426,7 +34427,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2898" s="4" t="inlineStr">
+      <c r="J2898" s="4" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -35139,7 +35140,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2960" s="24" t="inlineStr">
+      <c r="J2960" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -35164,7 +35165,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2961" s="24" t="inlineStr">
+      <c r="J2961" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -35237,7 +35238,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2966" s="24" t="inlineStr">
+      <c r="J2966" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -35390,7 +35391,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K2977" s="24" t="inlineStr">
+      <c r="J2977" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -35898,7 +35899,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3021" s="24" t="inlineStr">
+      <c r="J3021" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -35959,7 +35960,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3025" s="24" t="inlineStr">
+      <c r="J3025" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -35996,7 +35997,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3027" s="24" t="inlineStr">
+      <c r="J3027" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -36021,7 +36022,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3028" s="24" t="inlineStr">
+      <c r="J3028" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -36046,7 +36047,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3029" s="24" t="inlineStr">
+      <c r="J3029" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -37012,7 +37013,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3113" s="24" t="inlineStr">
+      <c r="J3113" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -37037,7 +37038,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3114" s="24" t="inlineStr">
+      <c r="J3114" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -37062,7 +37063,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3115" s="24" t="inlineStr">
+      <c r="J3115" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -37179,7 +37180,7 @@
         <v>700</v>
       </c>
       <c r="E3124" s="24" t="n"/>
-      <c r="K3124" s="24" t="inlineStr">
+      <c r="J3124" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -37204,7 +37205,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3125" s="24" t="inlineStr">
+      <c r="J3125" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -37241,7 +37242,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3127" s="24" t="inlineStr">
+      <c r="J3127" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -37266,7 +37267,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3128" s="24" t="inlineStr">
+      <c r="J3128" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -37291,7 +37292,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3129" s="24" t="inlineStr">
+      <c r="J3129" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -38667,7 +38668,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3249" s="24" t="inlineStr">
+      <c r="J3249" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -38692,7 +38693,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3250" s="24" t="inlineStr">
+      <c r="J3250" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -38753,7 +38754,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3254" s="24" t="inlineStr">
+      <c r="J3254" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -38802,7 +38803,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3257" s="24" t="inlineStr">
+      <c r="J3257" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -38839,7 +38840,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3259" s="24" t="inlineStr">
+      <c r="J3259" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -38888,7 +38889,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3262" s="24" t="inlineStr">
+      <c r="J3262" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -39646,7 +39647,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3341" s="24" t="inlineStr">
+      <c r="J3341" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -39679,7 +39680,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3343" s="24" t="inlineStr">
+      <c r="J3343" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -39722,7 +39723,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3346" s="24" t="inlineStr">
+      <c r="J3346" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -39745,7 +39746,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3347" s="24" t="inlineStr">
+      <c r="J3347" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -39768,7 +39769,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3348" s="24" t="inlineStr">
+      <c r="J3348" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -39811,7 +39812,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3351" s="24" t="inlineStr">
+      <c r="J3351" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -39864,7 +39865,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3355" s="24" t="inlineStr">
+      <c r="J3355" s="24" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -40778,7 +40779,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3435" t="inlineStr">
+      <c r="J3435" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -40815,7 +40816,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3437" t="inlineStr">
+      <c r="J3437" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -40924,7 +40925,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3445" t="inlineStr">
+      <c r="J3445" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -40961,7 +40962,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3447" t="inlineStr">
+      <c r="J3447" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -40986,7 +40987,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3448" t="inlineStr">
+      <c r="J3448" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -41035,7 +41036,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3451" t="inlineStr">
+      <c r="J3451" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -41060,7 +41061,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3452" t="inlineStr">
+      <c r="J3452" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -41749,7 +41750,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3512" t="inlineStr">
+      <c r="J3512" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -41786,7 +41787,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3514" t="inlineStr">
+      <c r="J3514" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -41811,7 +41812,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3515" t="inlineStr">
+      <c r="J3515" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -41836,7 +41837,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3516" t="inlineStr">
+      <c r="J3516" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -41861,7 +41862,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3517" t="inlineStr">
+      <c r="J3517" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -41898,7 +41899,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3519" t="inlineStr">
+      <c r="J3519" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -41923,7 +41924,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3520" t="inlineStr">
+      <c r="J3520" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -41972,7 +41973,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3523" t="inlineStr">
+      <c r="J3523" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -42009,7 +42010,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3525" t="inlineStr">
+      <c r="J3525" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -42034,7 +42035,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3526" t="inlineStr">
+      <c r="J3526" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -42071,7 +42072,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="K3528" t="inlineStr">
+      <c r="J3528" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -43374,7 +43375,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="L3641" s="7" t="inlineStr">
+      <c r="K3641" s="7" t="inlineStr">
         <is>
           <t>umgepflanzt</t>
         </is>
@@ -43399,7 +43400,7 @@
           <t>SYBA org</t>
         </is>
       </c>
-      <c r="L3642" s="7" t="inlineStr">
+      <c r="K3642" s="7" t="inlineStr">
         <is>
           <t>umgepflanzt</t>
         </is>
@@ -46779,8 +46780,7 @@
       <c r="G3920" s="24" t="n"/>
       <c r="H3920" s="24" t="n"/>
       <c r="I3920" s="24" t="n"/>
-      <c r="J3920" s="24" t="n"/>
-      <c r="K3920" t="inlineStr">
+      <c r="J3920" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -46821,8 +46821,7 @@
       <c r="G3922" s="24" t="n"/>
       <c r="H3922" s="24" t="n"/>
       <c r="I3922" s="24" t="n"/>
-      <c r="J3922" s="24" t="n"/>
-      <c r="K3922" t="inlineStr">
+      <c r="J3922" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -46851,8 +46850,7 @@
       <c r="G3923" s="24" t="n"/>
       <c r="H3923" s="24" t="n"/>
       <c r="I3923" s="24" t="n"/>
-      <c r="J3923" s="24" t="n"/>
-      <c r="K3923" t="inlineStr">
+      <c r="J3923" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -46881,8 +46879,7 @@
       <c r="G3924" s="24" t="n"/>
       <c r="H3924" s="24" t="n"/>
       <c r="I3924" s="24" t="n"/>
-      <c r="J3924" s="24" t="n"/>
-      <c r="K3924" t="inlineStr">
+      <c r="J3924" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -46947,8 +46944,7 @@
       <c r="G3928" s="24" t="n"/>
       <c r="H3928" s="24" t="n"/>
       <c r="I3928" s="24" t="n"/>
-      <c r="J3928" s="24" t="n"/>
-      <c r="K3928" t="inlineStr">
+      <c r="J3928" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -47025,8 +47021,7 @@
       <c r="G3933" s="24" t="n"/>
       <c r="H3933" s="24" t="n"/>
       <c r="I3933" s="24" t="n"/>
-      <c r="J3933" s="24" t="n"/>
-      <c r="K3933" t="inlineStr">
+      <c r="J3933" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -47067,8 +47062,7 @@
       <c r="G3935" s="24" t="n"/>
       <c r="H3935" s="24" t="n"/>
       <c r="I3935" s="24" t="n"/>
-      <c r="J3935" s="24" t="n"/>
-      <c r="K3935" t="inlineStr">
+      <c r="J3935" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -47097,8 +47091,7 @@
       <c r="G3936" s="24" t="n"/>
       <c r="H3936" s="24" t="n"/>
       <c r="I3936" s="24" t="n"/>
-      <c r="J3936" s="24" t="n"/>
-      <c r="K3936" t="inlineStr">
+      <c r="J3936" t="inlineStr">
         <is>
           <t>nematoden</t>
         </is>
@@ -64969,7 +64962,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="K5440" s="7" t="inlineStr">
+      <c r="J5440" s="7" t="inlineStr">
         <is>
           <t>bad, some pest bugs with black little shits</t>
         </is>
@@ -65196,7 +65189,7 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="K5456" s="7" t="inlineStr">
+      <c r="J5456" s="7" t="inlineStr">
         <is>
           <t>very bad, some pest bugs with black little shits</t>
         </is>
@@ -69504,6 +69497,8 @@
           <t xml:space="preserve">Philodendron Scandens Micans </t>
         </is>
       </c>
+      <c r="D5820" s="24" t="n"/>
+      <c r="E5820" s="24" t="n"/>
     </row>
     <row r="5821">
       <c r="A5821" t="inlineStr">
@@ -69516,6 +69511,8 @@
           <t>Scindapsus Treubii Moonlight</t>
         </is>
       </c>
+      <c r="D5821" s="24" t="n"/>
+      <c r="E5821" s="24" t="n"/>
     </row>
     <row r="5822">
       <c r="A5822" t="inlineStr">
@@ -69552,6 +69549,8 @@
           <t>Ficus Elastica Abidjan</t>
         </is>
       </c>
+      <c r="D5824" s="24" t="n"/>
+      <c r="E5824" s="24" t="n"/>
     </row>
     <row r="5825">
       <c r="A5825" t="inlineStr">
@@ -69600,6 +69599,8 @@
           <t>Sansevieria Laurentii</t>
         </is>
       </c>
+      <c r="D5828" s="24" t="n"/>
+      <c r="E5828" s="24" t="n"/>
     </row>
     <row r="5829">
       <c r="A5829" t="inlineStr">
@@ -69648,6 +69649,8 @@
           <t xml:space="preserve">Monstera Deliciosa </t>
         </is>
       </c>
+      <c r="D5832" s="24" t="n"/>
+      <c r="E5832" s="24" t="n"/>
     </row>
     <row r="5833">
       <c r="A5833" t="inlineStr">
@@ -69660,6 +69663,8 @@
           <t>Philodendron Imperial Red</t>
         </is>
       </c>
+      <c r="D5833" s="24" t="n"/>
+      <c r="E5833" s="24" t="n"/>
     </row>
     <row r="5834">
       <c r="A5834" t="inlineStr">
@@ -69672,6 +69677,8 @@
           <t>Philodendron McColleys Finale</t>
         </is>
       </c>
+      <c r="D5834" s="24" t="n"/>
+      <c r="E5834" s="24" t="n"/>
     </row>
     <row r="5835">
       <c r="A5835" t="inlineStr">
@@ -69684,6 +69691,8 @@
           <t>Philodendron Birkin</t>
         </is>
       </c>
+      <c r="D5835" s="24" t="n"/>
+      <c r="E5835" s="24" t="n"/>
     </row>
     <row r="5836">
       <c r="A5836" t="inlineStr">
@@ -69696,6 +69705,8 @@
           <t>Rhaphidophora Tetrasperma</t>
         </is>
       </c>
+      <c r="D5836" s="24" t="n"/>
+      <c r="E5836" s="24" t="n"/>
     </row>
     <row r="5837">
       <c r="A5837" t="inlineStr">
@@ -69711,10 +69722,8 @@
     </row>
     <row r="5838"/>
     <row r="5839">
-      <c r="A5839" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5839" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5839" t="inlineStr">
         <is>
@@ -69723,10 +69732,8 @@
       </c>
     </row>
     <row r="5840">
-      <c r="A5840" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5840" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5840" t="inlineStr">
         <is>
@@ -69735,10 +69742,8 @@
       </c>
     </row>
     <row r="5841">
-      <c r="A5841" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5841" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5841" t="inlineStr">
         <is>
@@ -69747,10 +69752,8 @@
       </c>
     </row>
     <row r="5842">
-      <c r="A5842" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5842" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5842" t="inlineStr">
         <is>
@@ -69759,10 +69762,8 @@
       </c>
     </row>
     <row r="5843">
-      <c r="A5843" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5843" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5843" t="inlineStr">
         <is>
@@ -69771,10 +69772,8 @@
       </c>
     </row>
     <row r="5844">
-      <c r="A5844" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5844" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5844" t="inlineStr">
         <is>
@@ -69783,10 +69782,8 @@
       </c>
     </row>
     <row r="5845">
-      <c r="A5845" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5845" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5845" t="inlineStr">
         <is>
@@ -69795,10 +69792,8 @@
       </c>
     </row>
     <row r="5846">
-      <c r="A5846" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5846" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5846" t="inlineStr">
         <is>
@@ -69807,10 +69802,8 @@
       </c>
     </row>
     <row r="5847">
-      <c r="A5847" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5847" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5847" t="inlineStr">
         <is>
@@ -69819,10 +69812,8 @@
       </c>
     </row>
     <row r="5848">
-      <c r="A5848" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5848" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5848" t="inlineStr">
         <is>
@@ -69831,10 +69822,8 @@
       </c>
     </row>
     <row r="5849">
-      <c r="A5849" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5849" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5849" t="inlineStr">
         <is>
@@ -69843,10 +69832,8 @@
       </c>
     </row>
     <row r="5850">
-      <c r="A5850" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5850" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5850" t="inlineStr">
         <is>
@@ -69855,10 +69842,8 @@
       </c>
     </row>
     <row r="5851">
-      <c r="A5851" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5851" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5851" t="inlineStr">
         <is>
@@ -69867,10 +69852,8 @@
       </c>
     </row>
     <row r="5852">
-      <c r="A5852" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5852" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5852" t="inlineStr">
         <is>
@@ -69879,10 +69862,8 @@
       </c>
     </row>
     <row r="5853">
-      <c r="A5853" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5853" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5853" t="inlineStr">
         <is>
@@ -69891,10 +69872,8 @@
       </c>
     </row>
     <row r="5854">
-      <c r="A5854" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5854" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5854" t="inlineStr">
         <is>
@@ -69903,10 +69882,8 @@
       </c>
     </row>
     <row r="5855">
-      <c r="A5855" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5855" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5855" t="inlineStr">
         <is>
@@ -69915,10 +69892,8 @@
       </c>
     </row>
     <row r="5856">
-      <c r="A5856" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5856" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5856" t="inlineStr">
         <is>
@@ -69927,10 +69902,8 @@
       </c>
     </row>
     <row r="5857">
-      <c r="A5857" t="inlineStr">
-        <is>
-          <t>17.04.2026</t>
-        </is>
+      <c r="A5857" s="2" t="n">
+        <v>46129</v>
       </c>
       <c r="B5857" t="inlineStr">
         <is>
@@ -69940,10 +69913,8 @@
     </row>
     <row r="5858"/>
     <row r="5859">
-      <c r="A5859" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5859" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5859" t="inlineStr">
         <is>
@@ -69952,10 +69923,8 @@
       </c>
     </row>
     <row r="5860">
-      <c r="A5860" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5860" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5860" t="inlineStr">
         <is>
@@ -69964,10 +69933,8 @@
       </c>
     </row>
     <row r="5861">
-      <c r="A5861" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5861" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5861" t="inlineStr">
         <is>
@@ -69976,10 +69943,8 @@
       </c>
     </row>
     <row r="5862">
-      <c r="A5862" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5862" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5862" t="inlineStr">
         <is>
@@ -69988,10 +69953,8 @@
       </c>
     </row>
     <row r="5863">
-      <c r="A5863" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5863" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5863" t="inlineStr">
         <is>
@@ -70000,10 +69963,8 @@
       </c>
     </row>
     <row r="5864">
-      <c r="A5864" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5864" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5864" t="inlineStr">
         <is>
@@ -70012,10 +69973,8 @@
       </c>
     </row>
     <row r="5865">
-      <c r="A5865" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5865" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5865" t="inlineStr">
         <is>
@@ -70024,10 +69983,8 @@
       </c>
     </row>
     <row r="5866">
-      <c r="A5866" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5866" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5866" t="inlineStr">
         <is>
@@ -70036,10 +69993,8 @@
       </c>
     </row>
     <row r="5867">
-      <c r="A5867" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5867" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5867" t="inlineStr">
         <is>
@@ -70048,10 +70003,8 @@
       </c>
     </row>
     <row r="5868">
-      <c r="A5868" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5868" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5868" t="inlineStr">
         <is>
@@ -70060,10 +70013,8 @@
       </c>
     </row>
     <row r="5869">
-      <c r="A5869" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5869" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5869" t="inlineStr">
         <is>
@@ -70072,10 +70023,8 @@
       </c>
     </row>
     <row r="5870">
-      <c r="A5870" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5870" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5870" t="inlineStr">
         <is>
@@ -70084,10 +70033,8 @@
       </c>
     </row>
     <row r="5871">
-      <c r="A5871" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5871" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5871" t="inlineStr">
         <is>
@@ -70096,10 +70043,8 @@
       </c>
     </row>
     <row r="5872">
-      <c r="A5872" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5872" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5872" t="inlineStr">
         <is>
@@ -70108,10 +70053,8 @@
       </c>
     </row>
     <row r="5873">
-      <c r="A5873" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5873" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5873" t="inlineStr">
         <is>
@@ -70120,10 +70063,8 @@
       </c>
     </row>
     <row r="5874">
-      <c r="A5874" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5874" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5874" t="inlineStr">
         <is>
@@ -70132,10 +70073,8 @@
       </c>
     </row>
     <row r="5875">
-      <c r="A5875" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5875" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5875" t="inlineStr">
         <is>
@@ -70144,10 +70083,8 @@
       </c>
     </row>
     <row r="5876">
-      <c r="A5876" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5876" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5876" t="inlineStr">
         <is>
@@ -70156,10 +70093,8 @@
       </c>
     </row>
     <row r="5877">
-      <c r="A5877" t="inlineStr">
-        <is>
-          <t>18.04.2026</t>
-        </is>
+      <c r="A5877" s="2" t="n">
+        <v>46130</v>
       </c>
       <c r="B5877" t="inlineStr">
         <is>
@@ -70169,22 +70104,26 @@
     </row>
     <row r="5878"/>
     <row r="5879">
-      <c r="A5879" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5879" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5879" t="inlineStr">
         <is>
           <t>Epipremnum Aureum</t>
         </is>
       </c>
+      <c r="D5879" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5879" s="24" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
     </row>
     <row r="5880">
-      <c r="A5880" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5880" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5880" t="inlineStr">
         <is>
@@ -70193,46 +70132,62 @@
       </c>
     </row>
     <row r="5881">
-      <c r="A5881" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5881" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5881" t="inlineStr">
         <is>
           <t>Scindapsus Treubii Moonlight</t>
         </is>
       </c>
+      <c r="D5881" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5881" s="24" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
     </row>
     <row r="5882">
-      <c r="A5882" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5882" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5882" t="inlineStr">
         <is>
           <t>Philodendron Hedaracium Brasil</t>
         </is>
       </c>
+      <c r="D5882" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5882" s="24" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
     </row>
     <row r="5883">
-      <c r="A5883" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5883" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5883" t="inlineStr">
         <is>
           <t>Monstera Adenossii</t>
         </is>
       </c>
+      <c r="D5883" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5883" s="24" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
     </row>
     <row r="5884">
-      <c r="A5884" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5884" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5884" t="inlineStr">
         <is>
@@ -70241,10 +70196,8 @@
       </c>
     </row>
     <row r="5885">
-      <c r="A5885" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5885" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5885" t="inlineStr">
         <is>
@@ -70253,22 +70206,26 @@
       </c>
     </row>
     <row r="5886">
-      <c r="A5886" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5886" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5886" t="inlineStr">
         <is>
           <t>Hoya Mathilde</t>
         </is>
       </c>
+      <c r="D5886" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5886" s="24" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
     </row>
     <row r="5887">
-      <c r="A5887" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5887" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5887" t="inlineStr">
         <is>
@@ -70277,10 +70234,8 @@
       </c>
     </row>
     <row r="5888">
-      <c r="A5888" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5888" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5888" t="inlineStr">
         <is>
@@ -70289,10 +70244,8 @@
       </c>
     </row>
     <row r="5889">
-      <c r="A5889" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5889" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5889" t="inlineStr">
         <is>
@@ -70301,22 +70254,26 @@
       </c>
     </row>
     <row r="5890">
-      <c r="A5890" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5890" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5890" t="inlineStr">
         <is>
           <t>Monstera Deliciosa Variegata</t>
         </is>
       </c>
+      <c r="D5890" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5890" s="24" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
     </row>
     <row r="5891">
-      <c r="A5891" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5891" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5891" t="inlineStr">
         <is>
@@ -70325,22 +70282,26 @@
       </c>
     </row>
     <row r="5892">
-      <c r="A5892" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5892" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5892" t="inlineStr">
         <is>
           <t xml:space="preserve">Monstera Deliciosa </t>
         </is>
       </c>
+      <c r="D5892" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5892" s="24" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
     </row>
     <row r="5893">
-      <c r="A5893" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5893" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5893" t="inlineStr">
         <is>
@@ -70348,91 +70309,132 @@
         </is>
       </c>
     </row>
-    <row r="5894">
-      <c r="A5894" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
-      </c>
-      <c r="B5894" t="inlineStr">
+    <row r="5894" customFormat="1" s="26">
+      <c r="A5894" s="25" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B5894" s="26" t="inlineStr">
         <is>
           <t>Philodendron McColleys Finale</t>
         </is>
       </c>
+      <c r="D5894" s="26" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5894" s="26" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
+      <c r="I5894" s="26" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
     </row>
     <row r="5895">
-      <c r="A5895" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
+      <c r="A5895" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5895" t="inlineStr">
         <is>
           <t>Philodendron Birkin</t>
         </is>
       </c>
-    </row>
-    <row r="5896">
-      <c r="A5896" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
-      </c>
-      <c r="B5896" t="inlineStr">
+      <c r="D5895" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5895" s="24" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
+    </row>
+    <row r="5896" customFormat="1" s="26">
+      <c r="A5896" s="25" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B5896" s="26" t="inlineStr">
         <is>
           <t>Rhaphidophora Tetrasperma</t>
         </is>
       </c>
-    </row>
-    <row r="5897">
-      <c r="A5897" t="inlineStr">
-        <is>
-          <t>19.04.2026</t>
-        </is>
-      </c>
-      <c r="B5897" t="inlineStr">
+      <c r="D5896" s="26" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5896" s="26" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
+      <c r="I5896" s="26" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="5897" customFormat="1" s="26">
+      <c r="A5897" s="25" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B5897" s="26" t="inlineStr">
         <is>
           <t>Philodendron Scandens Micans little</t>
         </is>
       </c>
-    </row>
-    <row r="5898"/>
-    <row r="5899">
-      <c r="A5899" t="inlineStr">
-        <is>
-          <t>20.04.2026</t>
-        </is>
+      <c r="D5897" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5897" s="24" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
+      <c r="I5897" s="26" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="5898" customFormat="1" s="26">
+      <c r="A5898" s="25" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B5898" s="26" t="inlineStr">
+        <is>
+          <t>Tradescantia zebrina</t>
+        </is>
+      </c>
+      <c r="D5898" s="24" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5898" s="24" t="inlineStr">
+        <is>
+          <t>SYBA org</t>
+        </is>
+      </c>
+    </row>
+    <row r="5899" customFormat="1" s="26">
+      <c r="A5899" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5899" t="inlineStr">
         <is>
-          <t>Epipremnum Aureum</t>
+          <t>Senecio rowleyanus</t>
         </is>
       </c>
     </row>
     <row r="5900">
-      <c r="A5900" t="inlineStr">
-        <is>
-          <t>20.04.2026</t>
-        </is>
+      <c r="A5900" s="2" t="n">
+        <v>46131</v>
       </c>
       <c r="B5900" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philodendron Scandens Micans </t>
-        </is>
-      </c>
-    </row>
-    <row r="5901">
-      <c r="A5901" t="inlineStr">
-        <is>
-          <t>20.04.2026</t>
-        </is>
-      </c>
-      <c r="B5901" t="inlineStr">
-        <is>
-          <t>Scindapsus Treubii Moonlight</t>
-        </is>
-      </c>
-    </row>
+          <t>Ledebouria socialis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5901"/>
     <row r="5902">
       <c r="A5902" t="inlineStr">
         <is>
@@ -70441,7 +70443,7 @@
       </c>
       <c r="B5902" t="inlineStr">
         <is>
-          <t>Philodendron Hedaracium Brasil</t>
+          <t>Epipremnum Aureum</t>
         </is>
       </c>
     </row>
@@ -70453,7 +70455,7 @@
       </c>
       <c r="B5903" t="inlineStr">
         <is>
-          <t>Monstera Adenossii</t>
+          <t xml:space="preserve">Philodendron Scandens Micans </t>
         </is>
       </c>
     </row>
@@ -70465,7 +70467,7 @@
       </c>
       <c r="B5904" t="inlineStr">
         <is>
-          <t>Ficus Elastica Abidjan</t>
+          <t>Scindapsus Treubii Moonlight</t>
         </is>
       </c>
     </row>
@@ -70477,7 +70479,7 @@
       </c>
       <c r="B5905" t="inlineStr">
         <is>
-          <t>Peperomia Hope</t>
+          <t>Philodendron Hedaracium Brasil</t>
         </is>
       </c>
     </row>
@@ -70489,7 +70491,7 @@
       </c>
       <c r="B5906" t="inlineStr">
         <is>
-          <t>Hoya Mathilde</t>
+          <t>Monstera Adenossii</t>
         </is>
       </c>
     </row>
@@ -70501,7 +70503,7 @@
       </c>
       <c r="B5907" t="inlineStr">
         <is>
-          <t>Epipremnum Pinnatum Blue</t>
+          <t>Ficus Elastica Abidjan</t>
         </is>
       </c>
     </row>
@@ -70513,7 +70515,7 @@
       </c>
       <c r="B5908" t="inlineStr">
         <is>
-          <t>Sansevieria Laurentii</t>
+          <t>Peperomia Hope</t>
         </is>
       </c>
     </row>
@@ -70525,7 +70527,7 @@
       </c>
       <c r="B5909" t="inlineStr">
         <is>
-          <t>Epipremnum Aureum Saal</t>
+          <t>Hoya Mathilde</t>
         </is>
       </c>
     </row>
@@ -70537,7 +70539,7 @@
       </c>
       <c r="B5910" t="inlineStr">
         <is>
-          <t>Monstera Deliciosa Variegata</t>
+          <t>Epipremnum Pinnatum Blue</t>
         </is>
       </c>
     </row>
@@ -70549,7 +70551,7 @@
       </c>
       <c r="B5911" t="inlineStr">
         <is>
-          <t>Pachira Aquatica</t>
+          <t>Sansevieria Laurentii</t>
         </is>
       </c>
     </row>
@@ -70561,7 +70563,7 @@
       </c>
       <c r="B5912" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monstera Deliciosa </t>
+          <t>Epipremnum Aureum Saal</t>
         </is>
       </c>
     </row>
@@ -70573,7 +70575,7 @@
       </c>
       <c r="B5913" t="inlineStr">
         <is>
-          <t>Philodendron Imperial Red</t>
+          <t>Monstera Deliciosa Variegata</t>
         </is>
       </c>
     </row>
@@ -70585,7 +70587,7 @@
       </c>
       <c r="B5914" t="inlineStr">
         <is>
-          <t>Philodendron McColleys Finale</t>
+          <t>Pachira Aquatica</t>
         </is>
       </c>
     </row>
@@ -70597,7 +70599,7 @@
       </c>
       <c r="B5915" t="inlineStr">
         <is>
-          <t>Philodendron Birkin</t>
+          <t xml:space="preserve">Monstera Deliciosa </t>
         </is>
       </c>
     </row>
@@ -70609,7 +70611,7 @@
       </c>
       <c r="B5916" t="inlineStr">
         <is>
-          <t>Rhaphidophora Tetrasperma</t>
+          <t>Philodendron Imperial Red</t>
         </is>
       </c>
     </row>
@@ -70621,125 +70623,83 @@
       </c>
       <c r="B5917" t="inlineStr">
         <is>
-          <t>Philodendron Scandens Micans little</t>
-        </is>
-      </c>
-    </row>
-    <row r="5918"/>
+          <t>Philodendron McColleys Finale</t>
+        </is>
+      </c>
+    </row>
+    <row r="5918">
+      <c r="A5918" t="inlineStr">
+        <is>
+          <t>20.04.2026</t>
+        </is>
+      </c>
+      <c r="B5918" t="inlineStr">
+        <is>
+          <t>Philodendron Birkin</t>
+        </is>
+      </c>
+    </row>
     <row r="5919">
       <c r="A5919" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>20.04.2026</t>
         </is>
       </c>
       <c r="B5919" t="inlineStr">
         <is>
-          <t>Epipremnum Aureum</t>
-        </is>
-      </c>
-      <c r="C5919" t="inlineStr"/>
-      <c r="D5919" t="inlineStr"/>
-      <c r="E5919" t="inlineStr"/>
-      <c r="F5919" t="inlineStr"/>
-      <c r="G5919" t="inlineStr"/>
-      <c r="H5919" t="inlineStr"/>
-      <c r="I5919" t="inlineStr"/>
+          <t>Rhaphidophora Tetrasperma</t>
+        </is>
+      </c>
     </row>
     <row r="5920">
       <c r="A5920" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>20.04.2026</t>
         </is>
       </c>
       <c r="B5920" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philodendron Scandens Micans </t>
-        </is>
-      </c>
-      <c r="C5920" t="inlineStr"/>
-      <c r="D5920" t="inlineStr"/>
-      <c r="E5920" t="inlineStr"/>
-      <c r="F5920" t="inlineStr"/>
-      <c r="G5920" t="inlineStr"/>
-      <c r="H5920" t="inlineStr"/>
-      <c r="I5920" t="inlineStr"/>
+          <t>Philodendron Scandens Micans little</t>
+        </is>
+      </c>
     </row>
     <row r="5921">
       <c r="A5921" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>20.04.2026</t>
         </is>
       </c>
       <c r="B5921" t="inlineStr">
         <is>
-          <t>Scindapsus Treubii Moonlight</t>
-        </is>
-      </c>
-      <c r="C5921" t="inlineStr"/>
-      <c r="D5921" t="inlineStr"/>
-      <c r="E5921" t="inlineStr"/>
-      <c r="F5921" t="inlineStr"/>
-      <c r="G5921" t="inlineStr"/>
-      <c r="H5921" t="inlineStr"/>
-      <c r="I5921" t="inlineStr"/>
+          <t>Tradescantia zebrina</t>
+        </is>
+      </c>
     </row>
     <row r="5922">
       <c r="A5922" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>20.04.2026</t>
         </is>
       </c>
       <c r="B5922" t="inlineStr">
         <is>
-          <t>Philodendron Hedaracium Brasil</t>
-        </is>
-      </c>
-      <c r="C5922" t="inlineStr"/>
-      <c r="D5922" t="inlineStr"/>
-      <c r="E5922" t="inlineStr"/>
-      <c r="F5922" t="inlineStr"/>
-      <c r="G5922" t="inlineStr"/>
-      <c r="H5922" t="inlineStr"/>
-      <c r="I5922" t="inlineStr"/>
+          <t>Senecio rowleyanus</t>
+        </is>
+      </c>
     </row>
     <row r="5923">
       <c r="A5923" t="inlineStr">
         <is>
-          <t>21.04.2026</t>
+          <t>20.04.2026</t>
         </is>
       </c>
       <c r="B5923" t="inlineStr">
         <is>
-          <t>Monstera Adenossii</t>
-        </is>
-      </c>
-      <c r="C5923" t="inlineStr"/>
-      <c r="D5923" t="inlineStr"/>
-      <c r="E5923" t="inlineStr"/>
-      <c r="F5923" t="inlineStr"/>
-      <c r="G5923" t="inlineStr"/>
-      <c r="H5923" t="inlineStr"/>
-      <c r="I5923" t="inlineStr"/>
-    </row>
-    <row r="5924">
-      <c r="A5924" t="inlineStr">
-        <is>
-          <t>21.04.2026</t>
-        </is>
-      </c>
-      <c r="B5924" t="inlineStr">
-        <is>
-          <t>Ficus Elastica Abidjan</t>
-        </is>
-      </c>
-      <c r="C5924" t="inlineStr"/>
-      <c r="D5924" t="inlineStr"/>
-      <c r="E5924" t="inlineStr"/>
-      <c r="F5924" t="inlineStr"/>
-      <c r="G5924" t="inlineStr"/>
-      <c r="H5924" t="inlineStr"/>
-      <c r="I5924" t="inlineStr"/>
-    </row>
+          <t>Ledebouria socialis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5924"/>
     <row r="5925">
       <c r="A5925" t="inlineStr">
         <is>
@@ -70748,16 +70708,9 @@
       </c>
       <c r="B5925" t="inlineStr">
         <is>
-          <t>Peperomia Hope</t>
-        </is>
-      </c>
-      <c r="C5925" t="inlineStr"/>
-      <c r="D5925" t="inlineStr"/>
-      <c r="E5925" t="inlineStr"/>
-      <c r="F5925" t="inlineStr"/>
-      <c r="G5925" t="inlineStr"/>
-      <c r="H5925" t="inlineStr"/>
-      <c r="I5925" t="inlineStr"/>
+          <t>Epipremnum Aureum</t>
+        </is>
+      </c>
     </row>
     <row r="5926">
       <c r="A5926" t="inlineStr">
@@ -70767,16 +70720,9 @@
       </c>
       <c r="B5926" t="inlineStr">
         <is>
-          <t>Hoya Mathilde</t>
-        </is>
-      </c>
-      <c r="C5926" t="inlineStr"/>
-      <c r="D5926" t="inlineStr"/>
-      <c r="E5926" t="inlineStr"/>
-      <c r="F5926" t="inlineStr"/>
-      <c r="G5926" t="inlineStr"/>
-      <c r="H5926" t="inlineStr"/>
-      <c r="I5926" t="inlineStr"/>
+          <t xml:space="preserve">Philodendron Scandens Micans </t>
+        </is>
+      </c>
     </row>
     <row r="5927">
       <c r="A5927" t="inlineStr">
@@ -70786,16 +70732,9 @@
       </c>
       <c r="B5927" t="inlineStr">
         <is>
-          <t>Epipremnum Pinnatum Blue</t>
-        </is>
-      </c>
-      <c r="C5927" t="inlineStr"/>
-      <c r="D5927" t="inlineStr"/>
-      <c r="E5927" t="inlineStr"/>
-      <c r="F5927" t="inlineStr"/>
-      <c r="G5927" t="inlineStr"/>
-      <c r="H5927" t="inlineStr"/>
-      <c r="I5927" t="inlineStr"/>
+          <t>Scindapsus Treubii Moonlight</t>
+        </is>
+      </c>
     </row>
     <row r="5928">
       <c r="A5928" t="inlineStr">
@@ -70805,16 +70744,9 @@
       </c>
       <c r="B5928" t="inlineStr">
         <is>
-          <t>Sansevieria Laurentii</t>
-        </is>
-      </c>
-      <c r="C5928" t="inlineStr"/>
-      <c r="D5928" t="inlineStr"/>
-      <c r="E5928" t="inlineStr"/>
-      <c r="F5928" t="inlineStr"/>
-      <c r="G5928" t="inlineStr"/>
-      <c r="H5928" t="inlineStr"/>
-      <c r="I5928" t="inlineStr"/>
+          <t>Philodendron Hedaracium Brasil</t>
+        </is>
+      </c>
     </row>
     <row r="5929">
       <c r="A5929" t="inlineStr">
@@ -70824,16 +70756,9 @@
       </c>
       <c r="B5929" t="inlineStr">
         <is>
-          <t>Epipremnum Aureum Saal</t>
-        </is>
-      </c>
-      <c r="C5929" t="inlineStr"/>
-      <c r="D5929" t="inlineStr"/>
-      <c r="E5929" t="inlineStr"/>
-      <c r="F5929" t="inlineStr"/>
-      <c r="G5929" t="inlineStr"/>
-      <c r="H5929" t="inlineStr"/>
-      <c r="I5929" t="inlineStr"/>
+          <t>Monstera Adenossii</t>
+        </is>
+      </c>
     </row>
     <row r="5930">
       <c r="A5930" t="inlineStr">
@@ -70843,16 +70768,9 @@
       </c>
       <c r="B5930" t="inlineStr">
         <is>
-          <t>Monstera Deliciosa Variegata</t>
-        </is>
-      </c>
-      <c r="C5930" t="inlineStr"/>
-      <c r="D5930" t="inlineStr"/>
-      <c r="E5930" t="inlineStr"/>
-      <c r="F5930" t="inlineStr"/>
-      <c r="G5930" t="inlineStr"/>
-      <c r="H5930" t="inlineStr"/>
-      <c r="I5930" t="inlineStr"/>
+          <t>Ficus Elastica Abidjan</t>
+        </is>
+      </c>
     </row>
     <row r="5931">
       <c r="A5931" t="inlineStr">
@@ -70862,16 +70780,9 @@
       </c>
       <c r="B5931" t="inlineStr">
         <is>
-          <t>Pachira Aquatica</t>
-        </is>
-      </c>
-      <c r="C5931" t="inlineStr"/>
-      <c r="D5931" t="inlineStr"/>
-      <c r="E5931" t="inlineStr"/>
-      <c r="F5931" t="inlineStr"/>
-      <c r="G5931" t="inlineStr"/>
-      <c r="H5931" t="inlineStr"/>
-      <c r="I5931" t="inlineStr"/>
+          <t>Peperomia Hope</t>
+        </is>
+      </c>
     </row>
     <row r="5932">
       <c r="A5932" t="inlineStr">
@@ -70881,16 +70792,9 @@
       </c>
       <c r="B5932" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monstera Deliciosa </t>
-        </is>
-      </c>
-      <c r="C5932" t="inlineStr"/>
-      <c r="D5932" t="inlineStr"/>
-      <c r="E5932" t="inlineStr"/>
-      <c r="F5932" t="inlineStr"/>
-      <c r="G5932" t="inlineStr"/>
-      <c r="H5932" t="inlineStr"/>
-      <c r="I5932" t="inlineStr"/>
+          <t>Hoya Mathilde</t>
+        </is>
+      </c>
     </row>
     <row r="5933">
       <c r="A5933" t="inlineStr">
@@ -70900,16 +70804,9 @@
       </c>
       <c r="B5933" t="inlineStr">
         <is>
-          <t>Philodendron Imperial Red</t>
-        </is>
-      </c>
-      <c r="C5933" t="inlineStr"/>
-      <c r="D5933" t="inlineStr"/>
-      <c r="E5933" t="inlineStr"/>
-      <c r="F5933" t="inlineStr"/>
-      <c r="G5933" t="inlineStr"/>
-      <c r="H5933" t="inlineStr"/>
-      <c r="I5933" t="inlineStr"/>
+          <t>Epipremnum Pinnatum Blue</t>
+        </is>
+      </c>
     </row>
     <row r="5934">
       <c r="A5934" t="inlineStr">
@@ -70919,16 +70816,9 @@
       </c>
       <c r="B5934" t="inlineStr">
         <is>
-          <t>Philodendron McColleys Finale</t>
-        </is>
-      </c>
-      <c r="C5934" t="inlineStr"/>
-      <c r="D5934" t="inlineStr"/>
-      <c r="E5934" t="inlineStr"/>
-      <c r="F5934" t="inlineStr"/>
-      <c r="G5934" t="inlineStr"/>
-      <c r="H5934" t="inlineStr"/>
-      <c r="I5934" t="inlineStr"/>
+          <t>Sansevieria Laurentii</t>
+        </is>
+      </c>
     </row>
     <row r="5935">
       <c r="A5935" t="inlineStr">
@@ -70938,16 +70828,9 @@
       </c>
       <c r="B5935" t="inlineStr">
         <is>
-          <t>Philodendron Birkin</t>
-        </is>
-      </c>
-      <c r="C5935" t="inlineStr"/>
-      <c r="D5935" t="inlineStr"/>
-      <c r="E5935" t="inlineStr"/>
-      <c r="F5935" t="inlineStr"/>
-      <c r="G5935" t="inlineStr"/>
-      <c r="H5935" t="inlineStr"/>
-      <c r="I5935" t="inlineStr"/>
+          <t>Epipremnum Aureum Saal</t>
+        </is>
+      </c>
     </row>
     <row r="5936">
       <c r="A5936" t="inlineStr">
@@ -70957,16 +70840,9 @@
       </c>
       <c r="B5936" t="inlineStr">
         <is>
-          <t>Rhaphidophora Tetrasperma</t>
-        </is>
-      </c>
-      <c r="C5936" t="inlineStr"/>
-      <c r="D5936" t="inlineStr"/>
-      <c r="E5936" t="inlineStr"/>
-      <c r="F5936" t="inlineStr"/>
-      <c r="G5936" t="inlineStr"/>
-      <c r="H5936" t="inlineStr"/>
-      <c r="I5936" t="inlineStr"/>
+          <t>Monstera Deliciosa Variegata</t>
+        </is>
+      </c>
     </row>
     <row r="5937">
       <c r="A5937" t="inlineStr">
@@ -70976,189 +70852,119 @@
       </c>
       <c r="B5937" t="inlineStr">
         <is>
-          <t>Philodendron Scandens Micans little</t>
-        </is>
-      </c>
-      <c r="C5937" t="inlineStr"/>
-      <c r="D5937" t="inlineStr"/>
-      <c r="E5937" t="inlineStr"/>
-      <c r="F5937" t="inlineStr"/>
-      <c r="G5937" t="inlineStr"/>
-      <c r="H5937" t="inlineStr"/>
-      <c r="I5937" t="inlineStr"/>
-    </row>
-    <row r="5938"/>
+          <t>Pachira Aquatica</t>
+        </is>
+      </c>
+    </row>
+    <row r="5938">
+      <c r="A5938" t="inlineStr">
+        <is>
+          <t>21.04.2026</t>
+        </is>
+      </c>
+      <c r="B5938" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monstera Deliciosa </t>
+        </is>
+      </c>
+    </row>
     <row r="5939">
       <c r="A5939" t="inlineStr">
         <is>
-          <t>22.04.2026</t>
+          <t>21.04.2026</t>
         </is>
       </c>
       <c r="B5939" t="inlineStr">
         <is>
-          <t>Epipremnum Aureum</t>
-        </is>
-      </c>
-      <c r="C5939" t="inlineStr"/>
-      <c r="D5939" t="inlineStr"/>
-      <c r="E5939" t="inlineStr"/>
-      <c r="F5939" t="inlineStr"/>
-      <c r="G5939" t="inlineStr"/>
-      <c r="H5939" t="inlineStr"/>
-      <c r="I5939" t="inlineStr"/>
+          <t>Philodendron Imperial Red</t>
+        </is>
+      </c>
     </row>
     <row r="5940">
       <c r="A5940" t="inlineStr">
         <is>
-          <t>22.04.2026</t>
+          <t>21.04.2026</t>
         </is>
       </c>
       <c r="B5940" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philodendron Scandens Micans </t>
-        </is>
-      </c>
-      <c r="C5940" t="inlineStr"/>
-      <c r="D5940" t="inlineStr"/>
-      <c r="E5940" t="inlineStr"/>
-      <c r="F5940" t="inlineStr"/>
-      <c r="G5940" t="inlineStr"/>
-      <c r="H5940" t="inlineStr"/>
-      <c r="I5940" t="inlineStr"/>
+          <t>Philodendron McColleys Finale</t>
+        </is>
+      </c>
     </row>
     <row r="5941">
       <c r="A5941" t="inlineStr">
         <is>
-          <t>22.04.2026</t>
+          <t>21.04.2026</t>
         </is>
       </c>
       <c r="B5941" t="inlineStr">
         <is>
-          <t>Scindapsus Treubii Moonlight</t>
-        </is>
-      </c>
-      <c r="C5941" t="inlineStr"/>
-      <c r="D5941" t="inlineStr"/>
-      <c r="E5941" t="inlineStr"/>
-      <c r="F5941" t="inlineStr"/>
-      <c r="G5941" t="inlineStr"/>
-      <c r="H5941" t="inlineStr"/>
-      <c r="I5941" t="inlineStr"/>
+          <t>Philodendron Birkin</t>
+        </is>
+      </c>
     </row>
     <row r="5942">
       <c r="A5942" t="inlineStr">
         <is>
-          <t>22.04.2026</t>
+          <t>21.04.2026</t>
         </is>
       </c>
       <c r="B5942" t="inlineStr">
         <is>
-          <t>Philodendron Hedaracium Brasil</t>
-        </is>
-      </c>
-      <c r="C5942" t="inlineStr"/>
-      <c r="D5942" t="inlineStr"/>
-      <c r="E5942" t="inlineStr"/>
-      <c r="F5942" t="inlineStr"/>
-      <c r="G5942" t="inlineStr"/>
-      <c r="H5942" t="inlineStr"/>
-      <c r="I5942" t="inlineStr"/>
+          <t>Rhaphidophora Tetrasperma</t>
+        </is>
+      </c>
     </row>
     <row r="5943">
       <c r="A5943" t="inlineStr">
         <is>
-          <t>22.04.2026</t>
+          <t>21.04.2026</t>
         </is>
       </c>
       <c r="B5943" t="inlineStr">
         <is>
-          <t>Monstera Adenossii</t>
-        </is>
-      </c>
-      <c r="C5943" t="inlineStr"/>
-      <c r="D5943" t="inlineStr"/>
-      <c r="E5943" t="inlineStr"/>
-      <c r="F5943" t="inlineStr"/>
-      <c r="G5943" t="inlineStr"/>
-      <c r="H5943" t="inlineStr"/>
-      <c r="I5943" t="inlineStr"/>
+          <t>Philodendron Scandens Micans little</t>
+        </is>
+      </c>
     </row>
     <row r="5944">
       <c r="A5944" t="inlineStr">
         <is>
-          <t>22.04.2026</t>
+          <t>21.04.2026</t>
         </is>
       </c>
       <c r="B5944" t="inlineStr">
         <is>
-          <t>Ficus Elastica Abidjan</t>
-        </is>
-      </c>
-      <c r="C5944" t="inlineStr"/>
-      <c r="D5944" t="inlineStr"/>
-      <c r="E5944" t="inlineStr"/>
-      <c r="F5944" t="inlineStr"/>
-      <c r="G5944" t="inlineStr"/>
-      <c r="H5944" t="inlineStr"/>
-      <c r="I5944" t="inlineStr"/>
+          <t>Tradescantia zebrina</t>
+        </is>
+      </c>
     </row>
     <row r="5945">
       <c r="A5945" t="inlineStr">
         <is>
-          <t>22.04.2026</t>
+          <t>21.04.2026</t>
         </is>
       </c>
       <c r="B5945" t="inlineStr">
         <is>
-          <t>Peperomia Hope</t>
-        </is>
-      </c>
-      <c r="C5945" t="inlineStr"/>
-      <c r="D5945" t="inlineStr"/>
-      <c r="E5945" t="inlineStr"/>
-      <c r="F5945" t="inlineStr"/>
-      <c r="G5945" t="inlineStr"/>
-      <c r="H5945" t="inlineStr"/>
-      <c r="I5945" t="inlineStr"/>
+          <t>Senecio rowleyanus</t>
+        </is>
+      </c>
     </row>
     <row r="5946">
       <c r="A5946" t="inlineStr">
         <is>
-          <t>22.04.2026</t>
+          <t>21.04.2026</t>
         </is>
       </c>
       <c r="B5946" t="inlineStr">
         <is>
-          <t>Hoya Mathilde</t>
-        </is>
-      </c>
-      <c r="C5946" t="inlineStr"/>
-      <c r="D5946" t="inlineStr"/>
-      <c r="E5946" t="inlineStr"/>
-      <c r="F5946" t="inlineStr"/>
-      <c r="G5946" t="inlineStr"/>
-      <c r="H5946" t="inlineStr"/>
-      <c r="I5946" t="inlineStr"/>
-    </row>
-    <row r="5947">
-      <c r="A5947" t="inlineStr">
-        <is>
-          <t>22.04.2026</t>
-        </is>
-      </c>
-      <c r="B5947" t="inlineStr">
-        <is>
-          <t>Epipremnum Pinnatum Blue</t>
-        </is>
-      </c>
-      <c r="C5947" t="inlineStr"/>
-      <c r="D5947" t="inlineStr"/>
-      <c r="E5947" t="inlineStr"/>
-      <c r="F5947" t="inlineStr"/>
-      <c r="G5947" t="inlineStr"/>
-      <c r="H5947" t="inlineStr"/>
-      <c r="I5947" t="inlineStr"/>
-    </row>
+          <t>Ledebouria socialis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5947"/>
     <row r="5948">
       <c r="A5948" t="inlineStr">
         <is>
@@ -71167,16 +70973,9 @@
       </c>
       <c r="B5948" t="inlineStr">
         <is>
-          <t>Sansevieria Laurentii</t>
-        </is>
-      </c>
-      <c r="C5948" t="inlineStr"/>
-      <c r="D5948" t="inlineStr"/>
-      <c r="E5948" t="inlineStr"/>
-      <c r="F5948" t="inlineStr"/>
-      <c r="G5948" t="inlineStr"/>
-      <c r="H5948" t="inlineStr"/>
-      <c r="I5948" t="inlineStr"/>
+          <t>Epipremnum Aureum</t>
+        </is>
+      </c>
     </row>
     <row r="5949">
       <c r="A5949" t="inlineStr">
@@ -71186,16 +70985,9 @@
       </c>
       <c r="B5949" t="inlineStr">
         <is>
-          <t>Epipremnum Aureum Saal</t>
-        </is>
-      </c>
-      <c r="C5949" t="inlineStr"/>
-      <c r="D5949" t="inlineStr"/>
-      <c r="E5949" t="inlineStr"/>
-      <c r="F5949" t="inlineStr"/>
-      <c r="G5949" t="inlineStr"/>
-      <c r="H5949" t="inlineStr"/>
-      <c r="I5949" t="inlineStr"/>
+          <t xml:space="preserve">Philodendron Scandens Micans </t>
+        </is>
+      </c>
     </row>
     <row r="5950">
       <c r="A5950" t="inlineStr">
@@ -71205,16 +70997,9 @@
       </c>
       <c r="B5950" t="inlineStr">
         <is>
-          <t>Monstera Deliciosa Variegata</t>
-        </is>
-      </c>
-      <c r="C5950" t="inlineStr"/>
-      <c r="D5950" t="inlineStr"/>
-      <c r="E5950" t="inlineStr"/>
-      <c r="F5950" t="inlineStr"/>
-      <c r="G5950" t="inlineStr"/>
-      <c r="H5950" t="inlineStr"/>
-      <c r="I5950" t="inlineStr"/>
+          <t>Scindapsus Treubii Moonlight</t>
+        </is>
+      </c>
     </row>
     <row r="5951">
       <c r="A5951" t="inlineStr">
@@ -71224,16 +71009,9 @@
       </c>
       <c r="B5951" t="inlineStr">
         <is>
-          <t>Pachira Aquatica</t>
-        </is>
-      </c>
-      <c r="C5951" t="inlineStr"/>
-      <c r="D5951" t="inlineStr"/>
-      <c r="E5951" t="inlineStr"/>
-      <c r="F5951" t="inlineStr"/>
-      <c r="G5951" t="inlineStr"/>
-      <c r="H5951" t="inlineStr"/>
-      <c r="I5951" t="inlineStr"/>
+          <t>Philodendron Hedaracium Brasil</t>
+        </is>
+      </c>
     </row>
     <row r="5952">
       <c r="A5952" t="inlineStr">
@@ -71243,16 +71021,9 @@
       </c>
       <c r="B5952" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monstera Deliciosa </t>
-        </is>
-      </c>
-      <c r="C5952" t="inlineStr"/>
-      <c r="D5952" t="inlineStr"/>
-      <c r="E5952" t="inlineStr"/>
-      <c r="F5952" t="inlineStr"/>
-      <c r="G5952" t="inlineStr"/>
-      <c r="H5952" t="inlineStr"/>
-      <c r="I5952" t="inlineStr"/>
+          <t>Monstera Adenossii</t>
+        </is>
+      </c>
     </row>
     <row r="5953">
       <c r="A5953" t="inlineStr">
@@ -71262,16 +71033,9 @@
       </c>
       <c r="B5953" t="inlineStr">
         <is>
-          <t>Philodendron Imperial Red</t>
-        </is>
-      </c>
-      <c r="C5953" t="inlineStr"/>
-      <c r="D5953" t="inlineStr"/>
-      <c r="E5953" t="inlineStr"/>
-      <c r="F5953" t="inlineStr"/>
-      <c r="G5953" t="inlineStr"/>
-      <c r="H5953" t="inlineStr"/>
-      <c r="I5953" t="inlineStr"/>
+          <t>Ficus Elastica Abidjan</t>
+        </is>
+      </c>
     </row>
     <row r="5954">
       <c r="A5954" t="inlineStr">
@@ -71281,16 +71045,9 @@
       </c>
       <c r="B5954" t="inlineStr">
         <is>
-          <t>Philodendron McColleys Finale</t>
-        </is>
-      </c>
-      <c r="C5954" t="inlineStr"/>
-      <c r="D5954" t="inlineStr"/>
-      <c r="E5954" t="inlineStr"/>
-      <c r="F5954" t="inlineStr"/>
-      <c r="G5954" t="inlineStr"/>
-      <c r="H5954" t="inlineStr"/>
-      <c r="I5954" t="inlineStr"/>
+          <t>Peperomia Hope</t>
+        </is>
+      </c>
     </row>
     <row r="5955">
       <c r="A5955" t="inlineStr">
@@ -71300,16 +71057,9 @@
       </c>
       <c r="B5955" t="inlineStr">
         <is>
-          <t>Philodendron Birkin</t>
-        </is>
-      </c>
-      <c r="C5955" t="inlineStr"/>
-      <c r="D5955" t="inlineStr"/>
-      <c r="E5955" t="inlineStr"/>
-      <c r="F5955" t="inlineStr"/>
-      <c r="G5955" t="inlineStr"/>
-      <c r="H5955" t="inlineStr"/>
-      <c r="I5955" t="inlineStr"/>
+          <t>Hoya Mathilde</t>
+        </is>
+      </c>
     </row>
     <row r="5956">
       <c r="A5956" t="inlineStr">
@@ -71319,16 +71069,9 @@
       </c>
       <c r="B5956" t="inlineStr">
         <is>
-          <t>Rhaphidophora Tetrasperma</t>
-        </is>
-      </c>
-      <c r="C5956" t="inlineStr"/>
-      <c r="D5956" t="inlineStr"/>
-      <c r="E5956" t="inlineStr"/>
-      <c r="F5956" t="inlineStr"/>
-      <c r="G5956" t="inlineStr"/>
-      <c r="H5956" t="inlineStr"/>
-      <c r="I5956" t="inlineStr"/>
+          <t>Epipremnum Pinnatum Blue</t>
+        </is>
+      </c>
     </row>
     <row r="5957">
       <c r="A5957" t="inlineStr">
@@ -71338,246 +71081,155 @@
       </c>
       <c r="B5957" t="inlineStr">
         <is>
-          <t>Philodendron Scandens Micans little</t>
-        </is>
-      </c>
-      <c r="C5957" t="inlineStr"/>
-      <c r="D5957" t="inlineStr"/>
-      <c r="E5957" t="inlineStr"/>
-      <c r="F5957" t="inlineStr"/>
-      <c r="G5957" t="inlineStr"/>
-      <c r="H5957" t="inlineStr"/>
-      <c r="I5957" t="inlineStr"/>
-    </row>
-    <row r="5958"/>
+          <t>Sansevieria Laurentii</t>
+        </is>
+      </c>
+    </row>
+    <row r="5958">
+      <c r="A5958" t="inlineStr">
+        <is>
+          <t>22.04.2026</t>
+        </is>
+      </c>
+      <c r="B5958" t="inlineStr">
+        <is>
+          <t>Epipremnum Aureum Saal</t>
+        </is>
+      </c>
+    </row>
     <row r="5959">
       <c r="A5959" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5959" t="inlineStr">
         <is>
-          <t>Epipremnum Aureum</t>
-        </is>
-      </c>
-      <c r="C5959" t="inlineStr"/>
-      <c r="D5959" t="inlineStr"/>
-      <c r="E5959" t="inlineStr"/>
-      <c r="F5959" t="inlineStr"/>
-      <c r="G5959" t="inlineStr"/>
-      <c r="H5959" t="inlineStr"/>
-      <c r="I5959" t="inlineStr"/>
+          <t>Monstera Deliciosa Variegata</t>
+        </is>
+      </c>
     </row>
     <row r="5960">
       <c r="A5960" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5960" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philodendron Scandens Micans </t>
-        </is>
-      </c>
-      <c r="C5960" t="inlineStr"/>
-      <c r="D5960" t="inlineStr"/>
-      <c r="E5960" t="inlineStr"/>
-      <c r="F5960" t="inlineStr"/>
-      <c r="G5960" t="inlineStr"/>
-      <c r="H5960" t="inlineStr"/>
-      <c r="I5960" t="inlineStr"/>
+          <t>Pachira Aquatica</t>
+        </is>
+      </c>
     </row>
     <row r="5961">
       <c r="A5961" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5961" t="inlineStr">
         <is>
-          <t>Scindapsus Treubii Moonlight</t>
-        </is>
-      </c>
-      <c r="C5961" t="inlineStr"/>
-      <c r="D5961" t="inlineStr"/>
-      <c r="E5961" t="inlineStr"/>
-      <c r="F5961" t="inlineStr"/>
-      <c r="G5961" t="inlineStr"/>
-      <c r="H5961" t="inlineStr"/>
-      <c r="I5961" t="inlineStr"/>
+          <t xml:space="preserve">Monstera Deliciosa </t>
+        </is>
+      </c>
     </row>
     <row r="5962">
       <c r="A5962" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5962" t="inlineStr">
         <is>
-          <t>Philodendron Hedaracium Brasil</t>
-        </is>
-      </c>
-      <c r="C5962" t="inlineStr"/>
-      <c r="D5962" t="inlineStr"/>
-      <c r="E5962" t="inlineStr"/>
-      <c r="F5962" t="inlineStr"/>
-      <c r="G5962" t="inlineStr"/>
-      <c r="H5962" t="inlineStr"/>
-      <c r="I5962" t="inlineStr"/>
+          <t>Philodendron Imperial Red</t>
+        </is>
+      </c>
     </row>
     <row r="5963">
       <c r="A5963" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5963" t="inlineStr">
         <is>
-          <t>Monstera Adenossii</t>
-        </is>
-      </c>
-      <c r="C5963" t="inlineStr"/>
-      <c r="D5963" t="inlineStr"/>
-      <c r="E5963" t="inlineStr"/>
-      <c r="F5963" t="inlineStr"/>
-      <c r="G5963" t="inlineStr"/>
-      <c r="H5963" t="inlineStr"/>
-      <c r="I5963" t="inlineStr"/>
+          <t>Philodendron McColleys Finale</t>
+        </is>
+      </c>
     </row>
     <row r="5964">
       <c r="A5964" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5964" t="inlineStr">
         <is>
-          <t>Ficus Elastica Abidjan</t>
-        </is>
-      </c>
-      <c r="C5964" t="inlineStr"/>
-      <c r="D5964" t="inlineStr"/>
-      <c r="E5964" t="inlineStr"/>
-      <c r="F5964" t="inlineStr"/>
-      <c r="G5964" t="inlineStr"/>
-      <c r="H5964" t="inlineStr"/>
-      <c r="I5964" t="inlineStr"/>
+          <t>Philodendron Birkin</t>
+        </is>
+      </c>
     </row>
     <row r="5965">
       <c r="A5965" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5965" t="inlineStr">
         <is>
-          <t>Peperomia Hope</t>
-        </is>
-      </c>
-      <c r="C5965" t="inlineStr"/>
-      <c r="D5965" t="inlineStr"/>
-      <c r="E5965" t="inlineStr"/>
-      <c r="F5965" t="inlineStr"/>
-      <c r="G5965" t="inlineStr"/>
-      <c r="H5965" t="inlineStr"/>
-      <c r="I5965" t="inlineStr"/>
+          <t>Rhaphidophora Tetrasperma</t>
+        </is>
+      </c>
     </row>
     <row r="5966">
       <c r="A5966" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5966" t="inlineStr">
         <is>
-          <t>Hoya Mathilde</t>
-        </is>
-      </c>
-      <c r="C5966" t="inlineStr"/>
-      <c r="D5966" t="inlineStr"/>
-      <c r="E5966" t="inlineStr"/>
-      <c r="F5966" t="inlineStr"/>
-      <c r="G5966" t="inlineStr"/>
-      <c r="H5966" t="inlineStr"/>
-      <c r="I5966" t="inlineStr"/>
+          <t>Philodendron Scandens Micans little</t>
+        </is>
+      </c>
     </row>
     <row r="5967">
       <c r="A5967" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5967" t="inlineStr">
         <is>
-          <t>Epipremnum Pinnatum Blue</t>
-        </is>
-      </c>
-      <c r="C5967" t="inlineStr"/>
-      <c r="D5967" t="inlineStr"/>
-      <c r="E5967" t="inlineStr"/>
-      <c r="F5967" t="inlineStr"/>
-      <c r="G5967" t="inlineStr"/>
-      <c r="H5967" t="inlineStr"/>
-      <c r="I5967" t="inlineStr"/>
+          <t>Tradescantia zebrina</t>
+        </is>
+      </c>
     </row>
     <row r="5968">
       <c r="A5968" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5968" t="inlineStr">
         <is>
-          <t>Sansevieria Laurentii</t>
-        </is>
-      </c>
-      <c r="C5968" t="inlineStr"/>
-      <c r="D5968" t="inlineStr"/>
-      <c r="E5968" t="inlineStr"/>
-      <c r="F5968" t="inlineStr"/>
-      <c r="G5968" t="inlineStr"/>
-      <c r="H5968" t="inlineStr"/>
-      <c r="I5968" t="inlineStr"/>
+          <t>Senecio rowleyanus</t>
+        </is>
+      </c>
     </row>
     <row r="5969">
       <c r="A5969" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>22.04.2026</t>
         </is>
       </c>
       <c r="B5969" t="inlineStr">
         <is>
-          <t>Epipremnum Aureum Saal</t>
-        </is>
-      </c>
-      <c r="C5969" t="inlineStr"/>
-      <c r="D5969" t="inlineStr"/>
-      <c r="E5969" t="inlineStr"/>
-      <c r="F5969" t="inlineStr"/>
-      <c r="G5969" t="inlineStr"/>
-      <c r="H5969" t="inlineStr"/>
-      <c r="I5969" t="inlineStr"/>
-    </row>
-    <row r="5970">
-      <c r="A5970" t="inlineStr">
-        <is>
-          <t>23.04.2026</t>
-        </is>
-      </c>
-      <c r="B5970" t="inlineStr">
-        <is>
-          <t>Monstera Deliciosa Variegata</t>
-        </is>
-      </c>
-      <c r="C5970" t="inlineStr"/>
-      <c r="D5970" t="inlineStr"/>
-      <c r="E5970" t="inlineStr"/>
-      <c r="F5970" t="inlineStr"/>
-      <c r="G5970" t="inlineStr"/>
-      <c r="H5970" t="inlineStr"/>
-      <c r="I5970" t="inlineStr"/>
-    </row>
+          <t>Ledebouria socialis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5970"/>
     <row r="5971">
       <c r="A5971" t="inlineStr">
         <is>
@@ -71586,16 +71238,9 @@
       </c>
       <c r="B5971" t="inlineStr">
         <is>
-          <t>Pachira Aquatica</t>
-        </is>
-      </c>
-      <c r="C5971" t="inlineStr"/>
-      <c r="D5971" t="inlineStr"/>
-      <c r="E5971" t="inlineStr"/>
-      <c r="F5971" t="inlineStr"/>
-      <c r="G5971" t="inlineStr"/>
-      <c r="H5971" t="inlineStr"/>
-      <c r="I5971" t="inlineStr"/>
+          <t>Epipremnum Aureum</t>
+        </is>
+      </c>
     </row>
     <row r="5972">
       <c r="A5972" t="inlineStr">
@@ -71605,16 +71250,9 @@
       </c>
       <c r="B5972" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monstera Deliciosa </t>
-        </is>
-      </c>
-      <c r="C5972" t="inlineStr"/>
-      <c r="D5972" t="inlineStr"/>
-      <c r="E5972" t="inlineStr"/>
-      <c r="F5972" t="inlineStr"/>
-      <c r="G5972" t="inlineStr"/>
-      <c r="H5972" t="inlineStr"/>
-      <c r="I5972" t="inlineStr"/>
+          <t xml:space="preserve">Philodendron Scandens Micans </t>
+        </is>
+      </c>
     </row>
     <row r="5973">
       <c r="A5973" t="inlineStr">
@@ -71624,16 +71262,9 @@
       </c>
       <c r="B5973" t="inlineStr">
         <is>
-          <t>Philodendron Imperial Red</t>
-        </is>
-      </c>
-      <c r="C5973" t="inlineStr"/>
-      <c r="D5973" t="inlineStr"/>
-      <c r="E5973" t="inlineStr"/>
-      <c r="F5973" t="inlineStr"/>
-      <c r="G5973" t="inlineStr"/>
-      <c r="H5973" t="inlineStr"/>
-      <c r="I5973" t="inlineStr"/>
+          <t>Scindapsus Treubii Moonlight</t>
+        </is>
+      </c>
     </row>
     <row r="5974">
       <c r="A5974" t="inlineStr">
@@ -71643,16 +71274,9 @@
       </c>
       <c r="B5974" t="inlineStr">
         <is>
-          <t>Philodendron McColleys Finale</t>
-        </is>
-      </c>
-      <c r="C5974" t="inlineStr"/>
-      <c r="D5974" t="inlineStr"/>
-      <c r="E5974" t="inlineStr"/>
-      <c r="F5974" t="inlineStr"/>
-      <c r="G5974" t="inlineStr"/>
-      <c r="H5974" t="inlineStr"/>
-      <c r="I5974" t="inlineStr"/>
+          <t>Philodendron Hedaracium Brasil</t>
+        </is>
+      </c>
     </row>
     <row r="5975">
       <c r="A5975" t="inlineStr">
@@ -71662,16 +71286,9 @@
       </c>
       <c r="B5975" t="inlineStr">
         <is>
-          <t>Philodendron Birkin</t>
-        </is>
-      </c>
-      <c r="C5975" t="inlineStr"/>
-      <c r="D5975" t="inlineStr"/>
-      <c r="E5975" t="inlineStr"/>
-      <c r="F5975" t="inlineStr"/>
-      <c r="G5975" t="inlineStr"/>
-      <c r="H5975" t="inlineStr"/>
-      <c r="I5975" t="inlineStr"/>
+          <t>Monstera Adenossii</t>
+        </is>
+      </c>
     </row>
     <row r="5976">
       <c r="A5976" t="inlineStr">
@@ -71681,16 +71298,9 @@
       </c>
       <c r="B5976" t="inlineStr">
         <is>
-          <t>Rhaphidophora Tetrasperma</t>
-        </is>
-      </c>
-      <c r="C5976" t="inlineStr"/>
-      <c r="D5976" t="inlineStr"/>
-      <c r="E5976" t="inlineStr"/>
-      <c r="F5976" t="inlineStr"/>
-      <c r="G5976" t="inlineStr"/>
-      <c r="H5976" t="inlineStr"/>
-      <c r="I5976" t="inlineStr"/>
+          <t>Ficus Elastica Abidjan</t>
+        </is>
+      </c>
     </row>
     <row r="5977">
       <c r="A5977" t="inlineStr">
@@ -71700,303 +71310,191 @@
       </c>
       <c r="B5977" t="inlineStr">
         <is>
-          <t>Philodendron Scandens Micans little</t>
-        </is>
-      </c>
-      <c r="C5977" t="inlineStr"/>
-      <c r="D5977" t="inlineStr"/>
-      <c r="E5977" t="inlineStr"/>
-      <c r="F5977" t="inlineStr"/>
-      <c r="G5977" t="inlineStr"/>
-      <c r="H5977" t="inlineStr"/>
-      <c r="I5977" t="inlineStr"/>
-    </row>
-    <row r="5978"/>
+          <t>Peperomia Hope</t>
+        </is>
+      </c>
+    </row>
+    <row r="5978">
+      <c r="A5978" t="inlineStr">
+        <is>
+          <t>23.04.2026</t>
+        </is>
+      </c>
+      <c r="B5978" t="inlineStr">
+        <is>
+          <t>Hoya Mathilde</t>
+        </is>
+      </c>
+    </row>
     <row r="5979">
       <c r="A5979" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5979" t="inlineStr">
         <is>
-          <t>Epipremnum Aureum</t>
-        </is>
-      </c>
-      <c r="C5979" t="inlineStr"/>
-      <c r="D5979" t="inlineStr"/>
-      <c r="E5979" t="inlineStr"/>
-      <c r="F5979" t="inlineStr"/>
-      <c r="G5979" t="inlineStr"/>
-      <c r="H5979" t="inlineStr"/>
-      <c r="I5979" t="inlineStr"/>
+          <t>Epipremnum Pinnatum Blue</t>
+        </is>
+      </c>
     </row>
     <row r="5980">
       <c r="A5980" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5980" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philodendron Scandens Micans </t>
-        </is>
-      </c>
-      <c r="C5980" t="inlineStr"/>
-      <c r="D5980" t="inlineStr"/>
-      <c r="E5980" t="inlineStr"/>
-      <c r="F5980" t="inlineStr"/>
-      <c r="G5980" t="inlineStr"/>
-      <c r="H5980" t="inlineStr"/>
-      <c r="I5980" t="inlineStr"/>
+          <t>Sansevieria Laurentii</t>
+        </is>
+      </c>
     </row>
     <row r="5981">
       <c r="A5981" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5981" t="inlineStr">
         <is>
-          <t>Scindapsus Treubii Moonlight</t>
-        </is>
-      </c>
-      <c r="C5981" t="inlineStr"/>
-      <c r="D5981" t="inlineStr"/>
-      <c r="E5981" t="inlineStr"/>
-      <c r="F5981" t="inlineStr"/>
-      <c r="G5981" t="inlineStr"/>
-      <c r="H5981" t="inlineStr"/>
-      <c r="I5981" t="inlineStr"/>
+          <t>Epipremnum Aureum Saal</t>
+        </is>
+      </c>
     </row>
     <row r="5982">
       <c r="A5982" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5982" t="inlineStr">
         <is>
-          <t>Philodendron Hedaracium Brasil</t>
-        </is>
-      </c>
-      <c r="C5982" t="inlineStr"/>
-      <c r="D5982" t="inlineStr"/>
-      <c r="E5982" t="inlineStr"/>
-      <c r="F5982" t="inlineStr"/>
-      <c r="G5982" t="inlineStr"/>
-      <c r="H5982" t="inlineStr"/>
-      <c r="I5982" t="inlineStr"/>
+          <t>Monstera Deliciosa Variegata</t>
+        </is>
+      </c>
     </row>
     <row r="5983">
       <c r="A5983" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5983" t="inlineStr">
         <is>
-          <t>Monstera Adenossii</t>
-        </is>
-      </c>
-      <c r="C5983" t="inlineStr"/>
-      <c r="D5983" t="inlineStr"/>
-      <c r="E5983" t="inlineStr"/>
-      <c r="F5983" t="inlineStr"/>
-      <c r="G5983" t="inlineStr"/>
-      <c r="H5983" t="inlineStr"/>
-      <c r="I5983" t="inlineStr"/>
+          <t>Pachira Aquatica</t>
+        </is>
+      </c>
     </row>
     <row r="5984">
       <c r="A5984" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5984" t="inlineStr">
         <is>
-          <t>Ficus Elastica Abidjan</t>
-        </is>
-      </c>
-      <c r="C5984" t="inlineStr"/>
-      <c r="D5984" t="inlineStr"/>
-      <c r="E5984" t="inlineStr"/>
-      <c r="F5984" t="inlineStr"/>
-      <c r="G5984" t="inlineStr"/>
-      <c r="H5984" t="inlineStr"/>
-      <c r="I5984" t="inlineStr"/>
+          <t xml:space="preserve">Monstera Deliciosa </t>
+        </is>
+      </c>
     </row>
     <row r="5985">
       <c r="A5985" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5985" t="inlineStr">
         <is>
-          <t>Peperomia Hope</t>
-        </is>
-      </c>
-      <c r="C5985" t="inlineStr"/>
-      <c r="D5985" t="inlineStr"/>
-      <c r="E5985" t="inlineStr"/>
-      <c r="F5985" t="inlineStr"/>
-      <c r="G5985" t="inlineStr"/>
-      <c r="H5985" t="inlineStr"/>
-      <c r="I5985" t="inlineStr"/>
+          <t>Philodendron Imperial Red</t>
+        </is>
+      </c>
     </row>
     <row r="5986">
       <c r="A5986" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5986" t="inlineStr">
         <is>
-          <t>Hoya Mathilde</t>
-        </is>
-      </c>
-      <c r="C5986" t="inlineStr"/>
-      <c r="D5986" t="inlineStr"/>
-      <c r="E5986" t="inlineStr"/>
-      <c r="F5986" t="inlineStr"/>
-      <c r="G5986" t="inlineStr"/>
-      <c r="H5986" t="inlineStr"/>
-      <c r="I5986" t="inlineStr"/>
+          <t>Philodendron McColleys Finale</t>
+        </is>
+      </c>
     </row>
     <row r="5987">
       <c r="A5987" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5987" t="inlineStr">
         <is>
-          <t>Epipremnum Pinnatum Blue</t>
-        </is>
-      </c>
-      <c r="C5987" t="inlineStr"/>
-      <c r="D5987" t="inlineStr"/>
-      <c r="E5987" t="inlineStr"/>
-      <c r="F5987" t="inlineStr"/>
-      <c r="G5987" t="inlineStr"/>
-      <c r="H5987" t="inlineStr"/>
-      <c r="I5987" t="inlineStr"/>
+          <t>Philodendron Birkin</t>
+        </is>
+      </c>
     </row>
     <row r="5988">
       <c r="A5988" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5988" t="inlineStr">
         <is>
-          <t>Sansevieria Laurentii</t>
-        </is>
-      </c>
-      <c r="C5988" t="inlineStr"/>
-      <c r="D5988" t="inlineStr"/>
-      <c r="E5988" t="inlineStr"/>
-      <c r="F5988" t="inlineStr"/>
-      <c r="G5988" t="inlineStr"/>
-      <c r="H5988" t="inlineStr"/>
-      <c r="I5988" t="inlineStr"/>
+          <t>Rhaphidophora Tetrasperma</t>
+        </is>
+      </c>
     </row>
     <row r="5989">
       <c r="A5989" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5989" t="inlineStr">
         <is>
-          <t>Epipremnum Aureum Saal</t>
-        </is>
-      </c>
-      <c r="C5989" t="inlineStr"/>
-      <c r="D5989" t="inlineStr"/>
-      <c r="E5989" t="inlineStr"/>
-      <c r="F5989" t="inlineStr"/>
-      <c r="G5989" t="inlineStr"/>
-      <c r="H5989" t="inlineStr"/>
-      <c r="I5989" t="inlineStr"/>
+          <t>Philodendron Scandens Micans little</t>
+        </is>
+      </c>
     </row>
     <row r="5990">
       <c r="A5990" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5990" t="inlineStr">
         <is>
-          <t>Monstera Deliciosa Variegata</t>
-        </is>
-      </c>
-      <c r="C5990" t="inlineStr"/>
-      <c r="D5990" t="inlineStr"/>
-      <c r="E5990" t="inlineStr"/>
-      <c r="F5990" t="inlineStr"/>
-      <c r="G5990" t="inlineStr"/>
-      <c r="H5990" t="inlineStr"/>
-      <c r="I5990" t="inlineStr"/>
+          <t>Tradescantia zebrina</t>
+        </is>
+      </c>
     </row>
     <row r="5991">
       <c r="A5991" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5991" t="inlineStr">
         <is>
-          <t>Pachira Aquatica</t>
-        </is>
-      </c>
-      <c r="C5991" t="inlineStr"/>
-      <c r="D5991" t="inlineStr"/>
-      <c r="E5991" t="inlineStr"/>
-      <c r="F5991" t="inlineStr"/>
-      <c r="G5991" t="inlineStr"/>
-      <c r="H5991" t="inlineStr"/>
-      <c r="I5991" t="inlineStr"/>
+          <t>Senecio rowleyanus</t>
+        </is>
+      </c>
     </row>
     <row r="5992">
       <c r="A5992" t="inlineStr">
         <is>
-          <t>24.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="B5992" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monstera Deliciosa </t>
-        </is>
-      </c>
-      <c r="C5992" t="inlineStr"/>
-      <c r="D5992" t="inlineStr"/>
-      <c r="E5992" t="inlineStr"/>
-      <c r="F5992" t="inlineStr"/>
-      <c r="G5992" t="inlineStr"/>
-      <c r="H5992" t="inlineStr"/>
-      <c r="I5992" t="inlineStr"/>
-    </row>
-    <row r="5993">
-      <c r="A5993" t="inlineStr">
-        <is>
-          <t>24.04.2026</t>
-        </is>
-      </c>
-      <c r="B5993" t="inlineStr">
-        <is>
-          <t>Philodendron Imperial Red</t>
-        </is>
-      </c>
-      <c r="C5993" t="inlineStr"/>
-      <c r="D5993" t="inlineStr"/>
-      <c r="E5993" t="inlineStr"/>
-      <c r="F5993" t="inlineStr"/>
-      <c r="G5993" t="inlineStr"/>
-      <c r="H5993" t="inlineStr"/>
-      <c r="I5993" t="inlineStr"/>
-    </row>
+          <t>Ledebouria socialis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5993"/>
     <row r="5994">
       <c r="A5994" t="inlineStr">
         <is>
@@ -72005,16 +71503,9 @@
       </c>
       <c r="B5994" t="inlineStr">
         <is>
-          <t>Philodendron McColleys Finale</t>
-        </is>
-      </c>
-      <c r="C5994" t="inlineStr"/>
-      <c r="D5994" t="inlineStr"/>
-      <c r="E5994" t="inlineStr"/>
-      <c r="F5994" t="inlineStr"/>
-      <c r="G5994" t="inlineStr"/>
-      <c r="H5994" t="inlineStr"/>
-      <c r="I5994" t="inlineStr"/>
+          <t>Epipremnum Aureum</t>
+        </is>
+      </c>
     </row>
     <row r="5995">
       <c r="A5995" t="inlineStr">
@@ -72024,16 +71515,9 @@
       </c>
       <c r="B5995" t="inlineStr">
         <is>
-          <t>Philodendron Birkin</t>
-        </is>
-      </c>
-      <c r="C5995" t="inlineStr"/>
-      <c r="D5995" t="inlineStr"/>
-      <c r="E5995" t="inlineStr"/>
-      <c r="F5995" t="inlineStr"/>
-      <c r="G5995" t="inlineStr"/>
-      <c r="H5995" t="inlineStr"/>
-      <c r="I5995" t="inlineStr"/>
+          <t xml:space="preserve">Philodendron Scandens Micans </t>
+        </is>
+      </c>
     </row>
     <row r="5996">
       <c r="A5996" t="inlineStr">
@@ -72043,16 +71527,9 @@
       </c>
       <c r="B5996" t="inlineStr">
         <is>
-          <t>Rhaphidophora Tetrasperma</t>
-        </is>
-      </c>
-      <c r="C5996" t="inlineStr"/>
-      <c r="D5996" t="inlineStr"/>
-      <c r="E5996" t="inlineStr"/>
-      <c r="F5996" t="inlineStr"/>
-      <c r="G5996" t="inlineStr"/>
-      <c r="H5996" t="inlineStr"/>
-      <c r="I5996" t="inlineStr"/>
+          <t>Scindapsus Treubii Moonlight</t>
+        </is>
+      </c>
     </row>
     <row r="5997">
       <c r="A5997" t="inlineStr">
@@ -72062,18 +71539,757 @@
       </c>
       <c r="B5997" t="inlineStr">
         <is>
+          <t>Philodendron Hedaracium Brasil</t>
+        </is>
+      </c>
+    </row>
+    <row r="5998">
+      <c r="A5998" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B5998" t="inlineStr">
+        <is>
+          <t>Monstera Adenossii</t>
+        </is>
+      </c>
+    </row>
+    <row r="5999">
+      <c r="A5999" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B5999" t="inlineStr">
+        <is>
+          <t>Ficus Elastica Abidjan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6000">
+      <c r="A6000" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6000" t="inlineStr">
+        <is>
+          <t>Peperomia Hope</t>
+        </is>
+      </c>
+    </row>
+    <row r="6001">
+      <c r="A6001" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6001" t="inlineStr">
+        <is>
+          <t>Hoya Mathilde</t>
+        </is>
+      </c>
+    </row>
+    <row r="6002">
+      <c r="A6002" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6002" t="inlineStr">
+        <is>
+          <t>Epipremnum Pinnatum Blue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6003">
+      <c r="A6003" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6003" t="inlineStr">
+        <is>
+          <t>Sansevieria Laurentii</t>
+        </is>
+      </c>
+    </row>
+    <row r="6004">
+      <c r="A6004" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6004" t="inlineStr">
+        <is>
+          <t>Epipremnum Aureum Saal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6005">
+      <c r="A6005" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6005" t="inlineStr">
+        <is>
+          <t>Monstera Deliciosa Variegata</t>
+        </is>
+      </c>
+    </row>
+    <row r="6006">
+      <c r="A6006" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6006" t="inlineStr">
+        <is>
+          <t>Pachira Aquatica</t>
+        </is>
+      </c>
+    </row>
+    <row r="6007">
+      <c r="A6007" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6007" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monstera Deliciosa </t>
+        </is>
+      </c>
+    </row>
+    <row r="6008">
+      <c r="A6008" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6008" t="inlineStr">
+        <is>
+          <t>Philodendron Imperial Red</t>
+        </is>
+      </c>
+    </row>
+    <row r="6009">
+      <c r="A6009" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6009" t="inlineStr">
+        <is>
+          <t>Philodendron McColleys Finale</t>
+        </is>
+      </c>
+    </row>
+    <row r="6010">
+      <c r="A6010" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6010" t="inlineStr">
+        <is>
+          <t>Philodendron Birkin</t>
+        </is>
+      </c>
+    </row>
+    <row r="6011">
+      <c r="A6011" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6011" t="inlineStr">
+        <is>
+          <t>Rhaphidophora Tetrasperma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6012">
+      <c r="A6012" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6012" t="inlineStr">
+        <is>
           <t>Philodendron Scandens Micans little</t>
         </is>
       </c>
-      <c r="C5997" t="inlineStr"/>
-      <c r="D5997" t="inlineStr"/>
-      <c r="E5997" t="inlineStr"/>
-      <c r="F5997" t="inlineStr"/>
-      <c r="G5997" t="inlineStr"/>
-      <c r="H5997" t="inlineStr"/>
-      <c r="I5997" t="inlineStr"/>
-    </row>
-    <row r="5998"/>
+    </row>
+    <row r="6013">
+      <c r="A6013" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6013" t="inlineStr">
+        <is>
+          <t>Tradescantia zebrina</t>
+        </is>
+      </c>
+    </row>
+    <row r="6014">
+      <c r="A6014" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6014" t="inlineStr">
+        <is>
+          <t>Senecio rowleyanus</t>
+        </is>
+      </c>
+    </row>
+    <row r="6015">
+      <c r="A6015" t="inlineStr">
+        <is>
+          <t>24.04.2026</t>
+        </is>
+      </c>
+      <c r="B6015" t="inlineStr">
+        <is>
+          <t>Ledebouria socialis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6016"/>
+    <row r="6017">
+      <c r="A6017" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6017" t="inlineStr">
+        <is>
+          <t>Epipremnum Aureum</t>
+        </is>
+      </c>
+    </row>
+    <row r="6018">
+      <c r="A6018" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6018" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philodendron Scandens Micans </t>
+        </is>
+      </c>
+    </row>
+    <row r="6019">
+      <c r="A6019" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6019" t="inlineStr">
+        <is>
+          <t>Scindapsus Treubii Moonlight</t>
+        </is>
+      </c>
+    </row>
+    <row r="6020">
+      <c r="A6020" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6020" t="inlineStr">
+        <is>
+          <t>Philodendron Hedaracium Brasil</t>
+        </is>
+      </c>
+    </row>
+    <row r="6021">
+      <c r="A6021" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6021" t="inlineStr">
+        <is>
+          <t>Monstera Adenossii</t>
+        </is>
+      </c>
+    </row>
+    <row r="6022">
+      <c r="A6022" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6022" t="inlineStr">
+        <is>
+          <t>Ficus Elastica Abidjan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6023">
+      <c r="A6023" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6023" t="inlineStr">
+        <is>
+          <t>Peperomia Hope</t>
+        </is>
+      </c>
+    </row>
+    <row r="6024">
+      <c r="A6024" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6024" t="inlineStr">
+        <is>
+          <t>Hoya Mathilde</t>
+        </is>
+      </c>
+    </row>
+    <row r="6025">
+      <c r="A6025" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6025" t="inlineStr">
+        <is>
+          <t>Epipremnum Pinnatum Blue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6026">
+      <c r="A6026" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6026" t="inlineStr">
+        <is>
+          <t>Sansevieria Laurentii</t>
+        </is>
+      </c>
+    </row>
+    <row r="6027">
+      <c r="A6027" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6027" t="inlineStr">
+        <is>
+          <t>Epipremnum Aureum Saal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6028">
+      <c r="A6028" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6028" t="inlineStr">
+        <is>
+          <t>Monstera Deliciosa Variegata</t>
+        </is>
+      </c>
+    </row>
+    <row r="6029">
+      <c r="A6029" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6029" t="inlineStr">
+        <is>
+          <t>Pachira Aquatica</t>
+        </is>
+      </c>
+    </row>
+    <row r="6030">
+      <c r="A6030" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6030" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monstera Deliciosa </t>
+        </is>
+      </c>
+    </row>
+    <row r="6031">
+      <c r="A6031" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6031" t="inlineStr">
+        <is>
+          <t>Philodendron Imperial Red</t>
+        </is>
+      </c>
+    </row>
+    <row r="6032">
+      <c r="A6032" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6032" t="inlineStr">
+        <is>
+          <t>Philodendron McColleys Finale</t>
+        </is>
+      </c>
+    </row>
+    <row r="6033">
+      <c r="A6033" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6033" t="inlineStr">
+        <is>
+          <t>Philodendron Birkin</t>
+        </is>
+      </c>
+    </row>
+    <row r="6034">
+      <c r="A6034" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6034" t="inlineStr">
+        <is>
+          <t>Rhaphidophora Tetrasperma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6035">
+      <c r="A6035" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6035" t="inlineStr">
+        <is>
+          <t>Philodendron Scandens Micans little</t>
+        </is>
+      </c>
+    </row>
+    <row r="6036">
+      <c r="A6036" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6036" t="inlineStr">
+        <is>
+          <t>Tradescantia zebrina</t>
+        </is>
+      </c>
+    </row>
+    <row r="6037">
+      <c r="A6037" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6037" t="inlineStr">
+        <is>
+          <t>Senecio rowleyanus</t>
+        </is>
+      </c>
+    </row>
+    <row r="6038">
+      <c r="A6038" t="inlineStr">
+        <is>
+          <t>25.04.2026</t>
+        </is>
+      </c>
+      <c r="B6038" t="inlineStr">
+        <is>
+          <t>Ledebouria socialis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6039"/>
+    <row r="6040">
+      <c r="A6040" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6040" t="inlineStr">
+        <is>
+          <t>Epipremnum Aureum</t>
+        </is>
+      </c>
+    </row>
+    <row r="6041">
+      <c r="A6041" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6041" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philodendron Scandens Micans </t>
+        </is>
+      </c>
+    </row>
+    <row r="6042">
+      <c r="A6042" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6042" t="inlineStr">
+        <is>
+          <t>Scindapsus Treubii Moonlight</t>
+        </is>
+      </c>
+    </row>
+    <row r="6043">
+      <c r="A6043" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6043" t="inlineStr">
+        <is>
+          <t>Philodendron Hedaracium Brasil</t>
+        </is>
+      </c>
+    </row>
+    <row r="6044">
+      <c r="A6044" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6044" t="inlineStr">
+        <is>
+          <t>Monstera Adenossii</t>
+        </is>
+      </c>
+    </row>
+    <row r="6045">
+      <c r="A6045" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6045" t="inlineStr">
+        <is>
+          <t>Ficus Elastica Abidjan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6046">
+      <c r="A6046" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6046" t="inlineStr">
+        <is>
+          <t>Peperomia Hope</t>
+        </is>
+      </c>
+    </row>
+    <row r="6047">
+      <c r="A6047" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6047" t="inlineStr">
+        <is>
+          <t>Hoya Mathilde</t>
+        </is>
+      </c>
+    </row>
+    <row r="6048">
+      <c r="A6048" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6048" t="inlineStr">
+        <is>
+          <t>Epipremnum Pinnatum Blue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6049">
+      <c r="A6049" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6049" t="inlineStr">
+        <is>
+          <t>Sansevieria Laurentii</t>
+        </is>
+      </c>
+    </row>
+    <row r="6050">
+      <c r="A6050" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6050" t="inlineStr">
+        <is>
+          <t>Epipremnum Aureum Saal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6051">
+      <c r="A6051" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6051" t="inlineStr">
+        <is>
+          <t>Monstera Deliciosa Variegata</t>
+        </is>
+      </c>
+    </row>
+    <row r="6052">
+      <c r="A6052" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6052" t="inlineStr">
+        <is>
+          <t>Pachira Aquatica</t>
+        </is>
+      </c>
+    </row>
+    <row r="6053">
+      <c r="A6053" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6053" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monstera Deliciosa </t>
+        </is>
+      </c>
+    </row>
+    <row r="6054">
+      <c r="A6054" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6054" t="inlineStr">
+        <is>
+          <t>Philodendron Imperial Red</t>
+        </is>
+      </c>
+    </row>
+    <row r="6055">
+      <c r="A6055" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6055" t="inlineStr">
+        <is>
+          <t>Philodendron McColleys Finale</t>
+        </is>
+      </c>
+    </row>
+    <row r="6056">
+      <c r="A6056" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6056" t="inlineStr">
+        <is>
+          <t>Philodendron Birkin</t>
+        </is>
+      </c>
+    </row>
+    <row r="6057">
+      <c r="A6057" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6057" t="inlineStr">
+        <is>
+          <t>Rhaphidophora Tetrasperma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6058">
+      <c r="A6058" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6058" t="inlineStr">
+        <is>
+          <t>Philodendron Scandens Micans little</t>
+        </is>
+      </c>
+    </row>
+    <row r="6059">
+      <c r="A6059" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6059" t="inlineStr">
+        <is>
+          <t>Tradescantia zebrina</t>
+        </is>
+      </c>
+    </row>
+    <row r="6060">
+      <c r="A6060" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6060" t="inlineStr">
+        <is>
+          <t>Senecio rowleyanus</t>
+        </is>
+      </c>
+    </row>
+    <row r="6061">
+      <c r="A6061" t="inlineStr">
+        <is>
+          <t>26.04.2026</t>
+        </is>
+      </c>
+      <c r="B6061" t="inlineStr">
+        <is>
+          <t>Ledebouria socialis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6062"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>